<commit_message>
Sort allComisiones to order careers and commissions alphabetically
</commit_message>
<xml_diff>
--- a/Presencialidad 2C 2026.xlsx
+++ b/Presencialidad 2C 2026.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="9000" tabRatio="500"/>
+    <workbookView windowWidth="27947" windowHeight="12240" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="133">
   <si>
     <t>Presencialidad 1C 2026</t>
   </si>
@@ -217,7 +217,7 @@
     <t>Inglés</t>
   </si>
   <si>
-    <t>Villariño</t>
+    <t>Vilariño</t>
   </si>
   <si>
     <t>Desarrollo de Sistemas Orientado a Objetos</t>
@@ -265,7 +265,7 @@
     <t>Taller de Comunicación</t>
   </si>
   <si>
-    <t>Litovisius</t>
+    <t>Litovicius</t>
   </si>
   <si>
     <t>PP3 Diseño de Arquitectura de Sistemas</t>
@@ -402,9 +402,6 @@
     <t>Técnicas de Procesamiento Digital de Imágenes</t>
   </si>
   <si>
-    <t>Vilariño</t>
-  </si>
-  <si>
     <t>Salico</t>
   </si>
   <si>
@@ -435,9 +432,6 @@
     <t>Metodología de Prueba de Sistemas</t>
   </si>
   <si>
-    <t>Litovicius</t>
-  </si>
-  <si>
     <t>Desarrollo de Aplicaciones para Dispositivos Móviles</t>
   </si>
   <si>
@@ -447,16 +441,16 @@
     <t>Ferraro</t>
   </si>
   <si>
+    <t>Desarrollo de Sistemas Web (Front End)</t>
+  </si>
+  <si>
+    <t>Uñates</t>
+  </si>
+  <si>
+    <t>Desarrollo e Implementación de Sistemas en la Nube</t>
+  </si>
+  <si>
     <t>Desarrollo de Sistemas Web (Back End)</t>
-  </si>
-  <si>
-    <t>Desarrollo de Sistemas Web (Front End)</t>
-  </si>
-  <si>
-    <t>Uñates</t>
-  </si>
-  <si>
-    <t>Desarrollo e Implementación de Sistemas en la Nube</t>
   </si>
   <si>
     <t>Campagna</t>
@@ -1102,13 +1096,17 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1116,6 +1114,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1460,6 +1459,22 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
     </row>
     <row r="2" spans="1:17">
       <c r="A2" s="2" t="s">
@@ -1518,16 +1533,28 @@
       <c r="A3" s="3">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="J3" t="s">
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
+      <c r="N3" s="1"/>
+      <c r="O3" s="1"/>
+      <c r="P3" s="1"/>
+      <c r="Q3" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1535,128 +1562,191 @@
       <c r="A4" s="3">
         <v>2</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="L4" t="s">
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="M4" t="s">
+      <c r="M4" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="O4" t="s">
+      <c r="N4" s="1"/>
+      <c r="O4" s="1" t="s">
         <v>20</v>
       </c>
+      <c r="P4" s="1"/>
+      <c r="Q4" s="1"/>
     </row>
     <row r="5" spans="1:17">
       <c r="A5" s="3">
         <v>3</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F5" t="s">
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H5" t="s">
+      <c r="G5" s="1"/>
+      <c r="H5" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="P5" t="s">
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+      <c r="O5" s="1"/>
+      <c r="P5" s="1" t="s">
         <v>20</v>
       </c>
+      <c r="Q5" s="1"/>
     </row>
     <row r="6" spans="1:17">
       <c r="A6" s="3">
         <v>4</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D6" t="s">
+      <c r="C6" s="1"/>
+      <c r="D6" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G6" t="s">
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1" t="s">
         <v>20</v>
       </c>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+      <c r="O6" s="1"/>
+      <c r="P6" s="1"/>
+      <c r="Q6" s="1"/>
     </row>
     <row r="7" spans="1:17">
       <c r="A7" s="3">
         <v>5</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="I7" t="s">
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K7" t="s">
+      <c r="J7" s="1"/>
+      <c r="K7" s="1" t="s">
         <v>20</v>
       </c>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="O7" s="1"/>
+      <c r="P7" s="1"/>
+      <c r="Q7" s="1"/>
     </row>
     <row r="8" spans="1:17">
       <c r="A8" s="3">
         <v>6</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E8" t="s">
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="N8" t="s">
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1" t="s">
         <v>19</v>
       </c>
+      <c r="O8" s="1"/>
+      <c r="P8" s="1"/>
+      <c r="Q8" s="1"/>
     </row>
     <row r="9" spans="1:17">
       <c r="A9" s="3">
         <v>7</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C9" t="s">
-        <v>28</v>
-      </c>
-      <c r="D9" t="s">
-        <v>28</v>
-      </c>
-      <c r="E9" t="s">
-        <v>28</v>
-      </c>
-      <c r="F9" t="s">
-        <v>28</v>
-      </c>
-      <c r="G9" t="s">
-        <v>28</v>
-      </c>
-      <c r="H9" t="s">
-        <v>28</v>
-      </c>
-      <c r="I9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J9" t="s">
-        <v>28</v>
-      </c>
-      <c r="K9" t="s">
-        <v>28</v>
-      </c>
-      <c r="L9" t="s">
-        <v>28</v>
-      </c>
-      <c r="M9" t="s">
-        <v>28</v>
-      </c>
-      <c r="N9" t="s">
-        <v>28</v>
-      </c>
-      <c r="O9" t="s">
-        <v>28</v>
-      </c>
-      <c r="P9" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q9" t="s">
+      <c r="C9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="M9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="N9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="P9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q9" s="1" t="s">
         <v>28</v>
       </c>
     </row>
@@ -1664,52 +1754,52 @@
       <c r="A10" s="3">
         <v>8</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C10" t="s">
-        <v>28</v>
-      </c>
-      <c r="D10" t="s">
-        <v>28</v>
-      </c>
-      <c r="E10" t="s">
-        <v>28</v>
-      </c>
-      <c r="F10" t="s">
-        <v>28</v>
-      </c>
-      <c r="G10" t="s">
-        <v>28</v>
-      </c>
-      <c r="H10" t="s">
-        <v>28</v>
-      </c>
-      <c r="I10" t="s">
-        <v>28</v>
-      </c>
-      <c r="J10" t="s">
-        <v>28</v>
-      </c>
-      <c r="K10" t="s">
-        <v>28</v>
-      </c>
-      <c r="L10" t="s">
-        <v>28</v>
-      </c>
-      <c r="M10" t="s">
-        <v>28</v>
-      </c>
-      <c r="N10" t="s">
-        <v>28</v>
-      </c>
-      <c r="O10" t="s">
-        <v>28</v>
-      </c>
-      <c r="P10" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q10" t="s">
+      <c r="C10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="N10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="P10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q10" s="1" t="s">
         <v>28</v>
       </c>
     </row>
@@ -1717,16 +1807,28 @@
       <c r="A11" s="3">
         <v>9</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="J11" t="s">
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="Q11" t="s">
+      <c r="K11" s="1"/>
+      <c r="L11" s="1"/>
+      <c r="M11" s="1"/>
+      <c r="N11" s="1"/>
+      <c r="O11" s="1"/>
+      <c r="P11" s="1"/>
+      <c r="Q11" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1734,128 +1836,191 @@
       <c r="A12" s="3">
         <v>10</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="L12" t="s">
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
+      <c r="K12" s="1"/>
+      <c r="L12" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="M12" t="s">
+      <c r="M12" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="O12" t="s">
+      <c r="N12" s="1"/>
+      <c r="O12" s="1" t="s">
         <v>20</v>
       </c>
+      <c r="P12" s="1"/>
+      <c r="Q12" s="1"/>
     </row>
     <row r="13" spans="1:17">
       <c r="A13" s="3">
         <v>11</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="F13" t="s">
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H13" t="s">
+      <c r="G13" s="1"/>
+      <c r="H13" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="P13" t="s">
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
+      <c r="K13" s="1"/>
+      <c r="L13" s="1"/>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
+      <c r="O13" s="1"/>
+      <c r="P13" s="1" t="s">
         <v>20</v>
       </c>
+      <c r="Q13" s="1"/>
     </row>
     <row r="14" spans="1:17">
       <c r="A14" s="3">
         <v>12</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D14" t="s">
+      <c r="C14" s="1"/>
+      <c r="D14" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G14" t="s">
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1" t="s">
         <v>20</v>
       </c>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
+      <c r="L14" s="1"/>
+      <c r="M14" s="1"/>
+      <c r="N14" s="1"/>
+      <c r="O14" s="1"/>
+      <c r="P14" s="1"/>
+      <c r="Q14" s="1"/>
     </row>
     <row r="15" spans="1:17">
       <c r="A15" s="3">
         <v>13</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="I15" t="s">
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K15" t="s">
+      <c r="J15" s="1"/>
+      <c r="K15" s="1" t="s">
         <v>20</v>
       </c>
+      <c r="L15" s="1"/>
+      <c r="M15" s="1"/>
+      <c r="N15" s="1"/>
+      <c r="O15" s="1"/>
+      <c r="P15" s="1"/>
+      <c r="Q15" s="1"/>
     </row>
     <row r="16" spans="1:17">
       <c r="A16" s="3">
         <v>14</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="E16" t="s">
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="N16" t="s">
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1" t="s">
         <v>19</v>
       </c>
+      <c r="O16" s="1"/>
+      <c r="P16" s="1"/>
+      <c r="Q16" s="1"/>
     </row>
     <row r="17" spans="1:17">
       <c r="A17" s="3">
         <v>15</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C17" t="s">
-        <v>28</v>
-      </c>
-      <c r="D17" t="s">
-        <v>28</v>
-      </c>
-      <c r="E17" t="s">
-        <v>28</v>
-      </c>
-      <c r="F17" t="s">
-        <v>28</v>
-      </c>
-      <c r="G17" t="s">
-        <v>28</v>
-      </c>
-      <c r="H17" t="s">
-        <v>28</v>
-      </c>
-      <c r="I17" t="s">
-        <v>28</v>
-      </c>
-      <c r="J17" t="s">
-        <v>28</v>
-      </c>
-      <c r="K17" t="s">
-        <v>28</v>
-      </c>
-      <c r="L17" t="s">
-        <v>28</v>
-      </c>
-      <c r="M17" t="s">
-        <v>28</v>
-      </c>
-      <c r="N17" t="s">
-        <v>28</v>
-      </c>
-      <c r="O17" t="s">
-        <v>28</v>
-      </c>
-      <c r="P17" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q17" t="s">
+      <c r="C17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="L17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="M17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="N17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="P17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q17" s="1" t="s">
         <v>28</v>
       </c>
     </row>
@@ -1863,52 +2028,52 @@
       <c r="A18" s="3">
         <v>16</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C18" t="s">
-        <v>28</v>
-      </c>
-      <c r="D18" t="s">
-        <v>28</v>
-      </c>
-      <c r="E18" t="s">
-        <v>28</v>
-      </c>
-      <c r="F18" t="s">
-        <v>28</v>
-      </c>
-      <c r="G18" t="s">
-        <v>28</v>
-      </c>
-      <c r="H18" t="s">
-        <v>28</v>
-      </c>
-      <c r="I18" t="s">
-        <v>28</v>
-      </c>
-      <c r="J18" t="s">
-        <v>28</v>
-      </c>
-      <c r="K18" t="s">
-        <v>28</v>
-      </c>
-      <c r="L18" t="s">
-        <v>28</v>
-      </c>
-      <c r="M18" t="s">
-        <v>28</v>
-      </c>
-      <c r="N18" t="s">
-        <v>28</v>
-      </c>
-      <c r="O18" t="s">
-        <v>28</v>
-      </c>
-      <c r="P18" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q18" t="s">
+      <c r="C18" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="L18" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="M18" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="N18" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O18" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="P18" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q18" s="1" t="s">
         <v>28</v>
       </c>
     </row>
@@ -1937,31 +2102,31 @@
       <c r="N20" s="6"/>
     </row>
     <row r="21" spans="1:17">
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="7" t="s">
         <v>43</v>
       </c>
       <c r="D21" t="s">
         <v>44</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="E21" s="7" t="s">
         <v>43</v>
       </c>
       <c r="F21" t="s">
         <v>44</v>
       </c>
-      <c r="G21" s="2" t="s">
+      <c r="G21" s="7" t="s">
         <v>43</v>
       </c>
       <c r="H21" t="s">
         <v>44</v>
       </c>
-      <c r="I21" s="2" t="s">
+      <c r="I21" s="7" t="s">
         <v>43</v>
       </c>
       <c r="J21" t="s">
         <v>44</v>
       </c>
-      <c r="K21" s="2" t="s">
+      <c r="K21" s="7" t="s">
         <v>43</v>
       </c>
       <c r="L21" t="s">
@@ -1969,7 +2134,7 @@
       </c>
     </row>
     <row r="22" spans="1:17">
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="7" t="s">
         <v>3</v>
       </c>
       <c r="C22" t="s">
@@ -1978,41 +2143,28 @@
       <c r="D22" t="s">
         <v>46</v>
       </c>
-      <c r="E22" t="s">
-        <v>47</v>
-      </c>
-      <c r="F22" s="7" t="s">
-        <v>48</v>
-      </c>
+      <c r="F22" s="8"/>
       <c r="G22" t="s">
         <v>47</v>
       </c>
-      <c r="H22" s="7" t="s">
+      <c r="H22" s="8" t="s">
         <v>48</v>
       </c>
       <c r="I22" t="s">
         <v>49</v>
       </c>
-      <c r="J22" s="7" t="s">
+      <c r="J22" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="K22" s="7" t="s">
+      <c r="K22" s="8" t="s">
         <v>51</v>
       </c>
       <c r="L22" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="23" spans="1:17">
-      <c r="E23" t="s">
-        <v>45</v>
-      </c>
-      <c r="F23" t="s">
-        <v>46</v>
-      </c>
-    </row>
     <row r="24" spans="1:17">
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="7" t="s">
         <v>4</v>
       </c>
       <c r="C24" t="s">
@@ -2036,7 +2188,7 @@
       <c r="I24" t="s">
         <v>59</v>
       </c>
-      <c r="J24" s="8" t="s">
+      <c r="J24" s="9" t="s">
         <v>60</v>
       </c>
       <c r="K24" t="s">
@@ -2047,7 +2199,7 @@
       </c>
     </row>
     <row r="25" spans="1:17">
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="7" t="s">
         <v>5</v>
       </c>
       <c r="C25" t="s">
@@ -2082,10 +2234,10 @@
       </c>
     </row>
     <row r="26" spans="1:17">
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C26" s="9" t="s">
         <v>73</v>
       </c>
       <c r="D26" t="s">
@@ -2103,7 +2255,7 @@
       <c r="H26" t="s">
         <v>78</v>
       </c>
-      <c r="I26" s="8" t="s">
+      <c r="I26" s="9" t="s">
         <v>79</v>
       </c>
       <c r="J26" t="s">
@@ -2117,7 +2269,7 @@
       </c>
     </row>
     <row r="27" spans="1:17">
-      <c r="E27" s="8" t="s">
+      <c r="E27" s="9" t="s">
         <v>73</v>
       </c>
       <c r="F27" t="s">
@@ -2131,7 +2283,7 @@
       </c>
     </row>
     <row r="28" spans="1:17">
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C28" t="s">
@@ -2174,7 +2326,7 @@
       </c>
     </row>
     <row r="30" spans="1:17">
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="7" t="s">
         <v>8</v>
       </c>
       <c r="C30" t="s">
@@ -2189,12 +2341,8 @@
       <c r="F30" t="s">
         <v>93</v>
       </c>
-      <c r="G30" t="s">
-        <v>94</v>
-      </c>
-      <c r="H30" t="s">
-        <v>46</v>
-      </c>
+      <c r="G30"/>
+      <c r="H30"/>
       <c r="I30" t="s">
         <v>92</v>
       </c>
@@ -2208,19 +2356,11 @@
         <v>46</v>
       </c>
     </row>
-    <row r="31" spans="1:17">
-      <c r="G31" t="s">
-        <v>67</v>
-      </c>
-      <c r="H31" t="s">
-        <v>93</v>
-      </c>
-    </row>
     <row r="32" spans="1:17">
-      <c r="B32" s="2" t="s">
+      <c r="B32" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C32" s="8" t="s">
+      <c r="C32" s="9" t="s">
         <v>95</v>
       </c>
       <c r="D32" t="s">
@@ -2252,7 +2392,7 @@
       </c>
     </row>
     <row r="33" spans="2:12">
-      <c r="B33" s="2" t="s">
+      <c r="B33" s="7" t="s">
         <v>10</v>
       </c>
       <c r="C33" t="s">
@@ -2261,7 +2401,7 @@
       <c r="D33" t="s">
         <v>76</v>
       </c>
-      <c r="E33" s="7" t="s">
+      <c r="E33" s="8" t="s">
         <v>100</v>
       </c>
       <c r="F33" t="s">
@@ -2270,7 +2410,7 @@
       <c r="G33" t="s">
         <v>63</v>
       </c>
-      <c r="H33" s="7" t="s">
+      <c r="H33" s="8" t="s">
         <v>102</v>
       </c>
       <c r="I33" t="s">
@@ -2279,7 +2419,7 @@
       <c r="J33" t="s">
         <v>104</v>
       </c>
-      <c r="K33" s="7" t="s">
+      <c r="K33" s="8" t="s">
         <v>100</v>
       </c>
       <c r="L33" t="s">
@@ -2287,7 +2427,7 @@
       </c>
     </row>
     <row r="34" spans="2:12">
-      <c r="E34" s="7" t="s">
+      <c r="E34" s="8" t="s">
         <v>105</v>
       </c>
       <c r="F34" t="s">
@@ -2295,7 +2435,7 @@
       </c>
     </row>
     <row r="35" spans="2:12">
-      <c r="B35" s="2" t="s">
+      <c r="B35" s="7" t="s">
         <v>11</v>
       </c>
       <c r="C35" t="s">
@@ -2338,7 +2478,7 @@
       </c>
     </row>
     <row r="37" spans="2:12">
-      <c r="B37" s="2" t="s">
+      <c r="B37" s="7" t="s">
         <v>12</v>
       </c>
       <c r="C37" t="s">
@@ -2353,37 +2493,31 @@
       <c r="H37" t="s">
         <v>112</v>
       </c>
-      <c r="I37" t="s">
-        <v>45</v>
-      </c>
-      <c r="J37" t="s">
-        <v>112</v>
-      </c>
     </row>
     <row r="38" spans="2:12">
-      <c r="B38" s="2" t="s">
+      <c r="B38" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C38" s="8" t="s">
-        <v>113</v>
+      <c r="C38" s="9" t="s">
+        <v>57</v>
       </c>
       <c r="D38" t="s">
         <v>46</v>
       </c>
       <c r="E38" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F38" t="s">
         <v>52</v>
       </c>
       <c r="G38" t="s">
-        <v>113</v>
+        <v>57</v>
       </c>
       <c r="H38" t="s">
         <v>46</v>
       </c>
       <c r="I38" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="J38" t="s">
         <v>93</v>
@@ -2397,42 +2531,42 @@
     </row>
     <row r="39" spans="2:12">
       <c r="G39" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H39" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="40" spans="2:12">
-      <c r="B40" s="2" t="s">
+      <c r="B40" s="7" t="s">
         <v>14</v>
       </c>
       <c r="C40" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D40" t="s">
         <v>56</v>
       </c>
       <c r="E40" t="s">
+        <v>116</v>
+      </c>
+      <c r="F40" t="s">
         <v>117</v>
       </c>
-      <c r="F40" t="s">
+      <c r="G40" t="s">
         <v>118</v>
-      </c>
-      <c r="G40" t="s">
-        <v>119</v>
       </c>
       <c r="H40" t="s">
         <v>54</v>
       </c>
       <c r="I40" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="J40" t="s">
         <v>58</v>
       </c>
       <c r="K40" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="L40" t="s">
         <v>62</v>
@@ -2440,50 +2574,50 @@
     </row>
     <row r="41" spans="2:12">
       <c r="K41" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="L41" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="42" ht="43.2" spans="2:12">
-      <c r="B42" s="2" t="s">
+      <c r="B42" s="7" t="s">
         <v>15</v>
       </c>
       <c r="C42" t="s">
         <v>77</v>
       </c>
-      <c r="D42" s="9" t="s">
-        <v>122</v>
+      <c r="D42" s="10" t="s">
+        <v>121</v>
       </c>
       <c r="E42" t="s">
         <v>100</v>
       </c>
       <c r="F42" t="s">
+        <v>122</v>
+      </c>
+      <c r="G42" t="s">
+        <v>73</v>
+      </c>
+      <c r="H42" t="s">
         <v>123</v>
-      </c>
-      <c r="G42" t="s">
-        <v>124</v>
-      </c>
-      <c r="H42" t="s">
-        <v>125</v>
       </c>
       <c r="I42" t="s">
         <v>77</v>
       </c>
       <c r="J42" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="K42" t="s">
-        <v>124</v>
+        <v>73</v>
       </c>
       <c r="L42" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="43" spans="2:12">
       <c r="G43" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="H43" t="s">
         <v>72</v>
@@ -2492,11 +2626,11 @@
         <v>100</v>
       </c>
       <c r="J43" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="44" spans="2:12">
-      <c r="B44" s="2" t="s">
+      <c r="B44" s="7" t="s">
         <v>16</v>
       </c>
       <c r="C44" t="s">
@@ -2505,51 +2639,39 @@
       <c r="D44" t="s">
         <v>70</v>
       </c>
-      <c r="E44" t="s">
-        <v>45</v>
-      </c>
-      <c r="F44" t="s">
+      <c r="G44" t="s">
+        <v>120</v>
+      </c>
+      <c r="H44" t="s">
+        <v>126</v>
+      </c>
+      <c r="I44" t="s">
+        <v>127</v>
+      </c>
+      <c r="J44" t="s">
         <v>128</v>
-      </c>
-      <c r="G44" t="s">
-        <v>121</v>
-      </c>
-      <c r="H44" t="s">
-        <v>129</v>
-      </c>
-      <c r="I44" t="s">
-        <v>130</v>
-      </c>
-      <c r="J44" t="s">
-        <v>131</v>
       </c>
       <c r="K44" t="s">
         <v>45</v>
       </c>
       <c r="L44" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="45" spans="2:12">
+      <c r="G45" t="s">
+        <v>127</v>
+      </c>
+      <c r="H45" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="45" spans="2:12">
-      <c r="E45" t="s">
-        <v>47</v>
-      </c>
-      <c r="F45" t="s">
-        <v>70</v>
-      </c>
-      <c r="G45" t="s">
+    <row r="46" spans="2:12">
+      <c r="B46" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C46" t="s">
         <v>130</v>
-      </c>
-      <c r="H45" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="46" spans="2:12">
-      <c r="B46" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C46" t="s">
-        <v>132</v>
       </c>
       <c r="D46" t="s">
         <v>86</v>
@@ -2558,12 +2680,12 @@
         <v>89</v>
       </c>
       <c r="F46" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="G46" t="s">
-        <v>134</v>
-      </c>
-      <c r="H46" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="H46" s="8" t="s">
         <v>80</v>
       </c>
       <c r="I46" t="s">

</xml_diff>